<commit_message>
USB Storage v1.0.0 지정
</commit_message>
<xml_diff>
--- a/data/0000001/샘플.xlsx
+++ b/data/0000001/샘플.xlsx
@@ -397,44 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>이름</v>
-      </c>
-      <c r="B1" t="str">
-        <v>점수</v>
-      </c>
-      <c r="C1" t="str">
-        <v>등급</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>홍길동</v>
-      </c>
-      <c r="B2">
-        <v>95</v>
-      </c>
-      <c r="C2" t="str">
-        <v>A</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>김철수</v>
-      </c>
-      <c r="B3">
-        <v>88</v>
-      </c>
-      <c r="C3" t="str">
-        <v>B</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>